<commit_message>
[DOCS][IRQ] Interrupt Service Register Map
</commit_message>
<xml_diff>
--- a/documentation/ARM_Bare_Metal_Multicore_Boot.xlsx
+++ b/documentation/ARM_Bare_Metal_Multicore_Boot.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QEMU_Cortex-A72\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D77F02-871F-41EF-BB1C-13924F972289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C33214E5-1066-406A-8F39-168A5D04607A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core_Registers" sheetId="1" r:id="rId1"/>
@@ -20,13 +20,14 @@
     <sheet name="Stack_Memory_Map" sheetId="3" r:id="rId5"/>
     <sheet name="SCTLR_EL1_Bits" sheetId="4" r:id="rId6"/>
     <sheet name="PSCI_Functions" sheetId="5" r:id="rId7"/>
+    <sheet name="Interrupt_Registers" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="500">
   <si>
     <t>ARM Cortex-A72/A76 Core Register Map</t>
   </si>
@@ -1091,6 +1092,474 @@
       </rPr>
       <t>(Will use software stubs in QEMU, real hardware on RP5)</t>
     </r>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Address / Access</t>
+  </si>
+  <si>
+    <t>Key Bits</t>
+  </si>
+  <si>
+    <t>Bit Position</t>
+  </si>
+  <si>
+    <t>What To Look For</t>
+  </si>
+  <si>
+    <t>Multiprocessor Affinity Register</t>
+  </si>
+  <si>
+    <t>CPU sys reg (read-only via mrs)</t>
+  </si>
+  <si>
+    <t>Identifies which core is executing — used in boot.S to assign per-core stacks</t>
+  </si>
+  <si>
+    <t>Aff0 (Core ID)</t>
+  </si>
+  <si>
+    <t>[7:0]</t>
+  </si>
+  <si>
+    <t>0=Core0, 1=Core1, 2=Core2, 3=Core3</t>
+  </si>
+  <si>
+    <t>Vector Base Address Register</t>
+  </si>
+  <si>
+    <t>CPU sys reg (write via msr)</t>
+  </si>
+  <si>
+    <t>Base address of the 2KB IVT — CPU jumps to VBAR + group_offset + type_offset on exception</t>
+  </si>
+  <si>
+    <t>Base address</t>
+  </si>
+  <si>
+    <t>[63:11]</t>
+  </si>
+  <si>
+    <t>Must be 2KB aligned — bits [10:0] must be zero</t>
+  </si>
+  <si>
+    <t>DAIF</t>
+  </si>
+  <si>
+    <t>Debug/SError/IRQ/FIQ Mask</t>
+  </si>
+  <si>
+    <t>CPU sys reg (msr daifclr/daifset)</t>
+  </si>
+  <si>
+    <t>CPU-level gate that blocks all IRQs regardless of GIC state</t>
+  </si>
+  <si>
+    <t>I (IRQ mask)</t>
+  </si>
+  <si>
+    <t>Bit 7</t>
+  </si>
+  <si>
+    <t>0 = IRQs pass through, 1 = all IRQs blocked at CPU</t>
+  </si>
+  <si>
+    <t>ELR_EL1</t>
+  </si>
+  <si>
+    <t>Exception Link Register</t>
+  </si>
+  <si>
+    <t>CPU sys reg (auto-written by HW on exception)</t>
+  </si>
+  <si>
+    <t>Return address — holds PC of the interrupted instruction, restored by eret</t>
+  </si>
+  <si>
+    <t>Full PC</t>
+  </si>
+  <si>
+    <t>[63:0]</t>
+  </si>
+  <si>
+    <t>The exact instruction to resume after handler completes</t>
+  </si>
+  <si>
+    <t>SPSR_EL1</t>
+  </si>
+  <si>
+    <t>Saved Program Status Register</t>
+  </si>
+  <si>
+    <t>Snapshot of PSTATE at moment of interrupt — eret restores it atomically</t>
+  </si>
+  <si>
+    <t>M[3:0] (EL/SP mode)</t>
+  </si>
+  <si>
+    <t>[3:0]</t>
+  </si>
+  <si>
+    <t>0b0101 = EL1h (your normal state: EL1 with SP_EL1)</t>
+  </si>
+  <si>
+    <t>I (saved IRQ mask)</t>
+  </si>
+  <si>
+    <t>0 = IRQs were enabled before interrupt — eret will re-enable them</t>
+  </si>
+  <si>
+    <t>NZCV (condition flags)</t>
+  </si>
+  <si>
+    <t>[31:28]</t>
+  </si>
+  <si>
+    <t>Saved ALU flags — must be restored so interrupted code logic is correct</t>
+  </si>
+  <si>
+    <t>SP_EL1</t>
+  </si>
+  <si>
+    <t>Stack Pointer (EL1)</t>
+  </si>
+  <si>
+    <t>CPU sys reg (mov sp)</t>
+  </si>
+  <si>
+    <t>Per-core stack pointer — save_regs subtracts 272 bytes, restore_regs adds them back</t>
+  </si>
+  <si>
+    <t>Full address</t>
+  </si>
+  <si>
+    <t>Must be 16-byte aligned; grows downward; Core0 = 0x40204000</t>
+  </si>
+  <si>
+    <t>GICD_CTLR</t>
+  </si>
+  <si>
+    <t>GIC Distributor Control</t>
+  </si>
+  <si>
+    <t>0x08000000</t>
+  </si>
+  <si>
+    <t>Master on/off switch for the entire GIC distributor</t>
+  </si>
+  <si>
+    <t>EnableGrp0</t>
+  </si>
+  <si>
+    <t>Bit 0</t>
+  </si>
+  <si>
+    <t>1 = distributor forwards interrupts, 0 = all blocked</t>
+  </si>
+  <si>
+    <t>GICD_ISENABLER(n)</t>
+  </si>
+  <si>
+    <t>Interrupt Set-Enable</t>
+  </si>
+  <si>
+    <t>0x08000100 + n*4</t>
+  </si>
+  <si>
+    <t>Unmask one specific INTID — write 1 to the INTID's bit to enable it</t>
+  </si>
+  <si>
+    <t>Bit per INTID</t>
+  </si>
+  <si>
+    <t>Bit [INTID % 32]</t>
+  </si>
+  <si>
+    <t>Timer=bit30 in reg0 (0x40000000), UART=bit1 in reg1 (0x02)</t>
+  </si>
+  <si>
+    <t>GICD_ICENABLER(n)</t>
+  </si>
+  <si>
+    <t>Interrupt Clear-Enable</t>
+  </si>
+  <si>
+    <t>0x08000180 + n*4</t>
+  </si>
+  <si>
+    <t>Mask one specific INTID — write 1 to disable, write 0 does nothing</t>
+  </si>
+  <si>
+    <t>0xFFFFFFFF = mask all 32 INTIDs in that register</t>
+  </si>
+  <si>
+    <t>GICD_IPRIORITYR(n)</t>
+  </si>
+  <si>
+    <t>Interrupt Priority</t>
+  </si>
+  <si>
+    <t>0x08000400 + n*4</t>
+  </si>
+  <si>
+    <t>Set priority per INTID — lower number = higher urgency. 4 INTIDs packed per register</t>
+  </si>
+  <si>
+    <t>1 byte per INTID</t>
+  </si>
+  <si>
+    <t>[7:0] per byte</t>
+  </si>
+  <si>
+    <t>Your value 0xA0 = medium priority; must be &lt; GICC_PMR to pass</t>
+  </si>
+  <si>
+    <t>GICD_ITARGETSR(n)</t>
+  </si>
+  <si>
+    <t>Interrupt Target</t>
+  </si>
+  <si>
+    <t>0x08000800 + n*4</t>
+  </si>
+  <si>
+    <t>Route each INTID to specific CPU core(s). 4 INTIDs packed per register</t>
+  </si>
+  <si>
+    <t>Bit0=CPU0, Bit1=CPU1</t>
+  </si>
+  <si>
+    <t>0x01 = route to Core 0 only</t>
+  </si>
+  <si>
+    <t>GICD_ICFGR(n)</t>
+  </si>
+  <si>
+    <t>Interrupt Configuration</t>
+  </si>
+  <si>
+    <t>0x08000C00 + n*4</t>
+  </si>
+  <si>
+    <t>Level-sensitive vs edge-triggered. 2 bits per INTID</t>
+  </si>
+  <si>
+    <t>2 bits per INTID</t>
+  </si>
+  <si>
+    <t>Bit [2k+1]</t>
+  </si>
+  <si>
+    <t>0 = level-sensitive (your config), 1 = edge-triggered</t>
+  </si>
+  <si>
+    <t>GICC_CTLR</t>
+  </si>
+  <si>
+    <t>GIC CPU Interface Control</t>
+  </si>
+  <si>
+    <t>0x08010000</t>
+  </si>
+  <si>
+    <t>Enable the GIC-to-CPU signaling path — without this the CPU never sees IRQ</t>
+  </si>
+  <si>
+    <t>1 = GIC can assert IRQ line to this core</t>
+  </si>
+  <si>
+    <t>GICC_PMR</t>
+  </si>
+  <si>
+    <t>Priority Mask Register</t>
+  </si>
+  <si>
+    <t>0x08010004</t>
+  </si>
+  <si>
+    <t>Priority filter — only interrupts with priority value LOWER than PMR pass through</t>
+  </si>
+  <si>
+    <t>Priority threshold</t>
+  </si>
+  <si>
+    <t>0xFF = allow everything; your INTID priority 0xA0 &lt; 0xFF so it passes</t>
+  </si>
+  <si>
+    <t>GICC_BPR</t>
+  </si>
+  <si>
+    <t>Binary Point Register</t>
+  </si>
+  <si>
+    <t>0x08010008</t>
+  </si>
+  <si>
+    <t>Splits priority byte into group/subgroup — controls preemption granularity</t>
+  </si>
+  <si>
+    <t>Binary point</t>
+  </si>
+  <si>
+    <t>[2:0]</t>
+  </si>
+  <si>
+    <t>0 = no subpriority, all 8 bits are group priority</t>
+  </si>
+  <si>
+    <t>GICC_IAR</t>
+  </si>
+  <si>
+    <t>Interrupt Acknowledge Register</t>
+  </si>
+  <si>
+    <t>0x0801000C (read-only, destructive)</t>
+  </si>
+  <si>
+    <t>ACK the interrupt AND get the INTID in one read — transitions INTID pending→active</t>
+  </si>
+  <si>
+    <t>INTID</t>
+  </si>
+  <si>
+    <t>[9:0]</t>
+  </si>
+  <si>
+    <t>30=Timer, 33=UART0, 1023=spurious (ignore)</t>
+  </si>
+  <si>
+    <t>CPUID</t>
+  </si>
+  <si>
+    <t>[12:10]</t>
+  </si>
+  <si>
+    <t>Source CPU for SGIs — irrelevant for Timer/UART (PPI/SPI)</t>
+  </si>
+  <si>
+    <t>GICC_EOIR</t>
+  </si>
+  <si>
+    <t>End Of Interrupt Register</t>
+  </si>
+  <si>
+    <t>0x08010010 (write-only)</t>
+  </si>
+  <si>
+    <t>Signal handler completion — write full iar value back. Transitions INTID active→idle</t>
+  </si>
+  <si>
+    <t>Must write full iar</t>
+  </si>
+  <si>
+    <t>[12:0]</t>
+  </si>
+  <si>
+    <t>Forgetting EOIR = INTID stuck active forever, no more IRQs</t>
+  </si>
+  <si>
+    <t>UART_DR</t>
+  </si>
+  <si>
+    <t>UART Data Register</t>
+  </si>
+  <si>
+    <t>0x09000000 (QEMU) / 0x40030000 (RPi5)</t>
+  </si>
+  <si>
+    <t>Write to transmit a char, read to receive a char from FIFO</t>
+  </si>
+  <si>
+    <t>DATA (the ASCII byte)</t>
+  </si>
+  <si>
+    <t>0x41='A', 0x0D=Enter, 0x03=Ctrl+C, 0x1B=ESC</t>
+  </si>
+  <si>
+    <t>UART_FR</t>
+  </si>
+  <si>
+    <t>UART Flag Register</t>
+  </si>
+  <si>
+    <t>0x09000018 (QEMU) / 0x40030018 (RPi5)</t>
+  </si>
+  <si>
+    <t>FIFO status flags — check before reading or writing DR</t>
+  </si>
+  <si>
+    <t>RXFE (RX FIFO Empty)</t>
+  </si>
+  <si>
+    <t>Bit 4</t>
+  </si>
+  <si>
+    <t>0 = data available (uart_has_data returns true)</t>
+  </si>
+  <si>
+    <t>TXFF (TX FIFO Full)</t>
+  </si>
+  <si>
+    <t>Bit 5</t>
+  </si>
+  <si>
+    <t>0 = ready to send (uart_putc proceeds)</t>
+  </si>
+  <si>
+    <t>UART_IMSC</t>
+  </si>
+  <si>
+    <t>Interrupt Mask Set/Clear</t>
+  </si>
+  <si>
+    <t>0x09000038 (QEMU) / 0x40030038 (RPi5)</t>
+  </si>
+  <si>
+    <t>Unmask specific UART interrupt sources so PL011 asserts IRQ line to GIC</t>
+  </si>
+  <si>
+    <t>RXIM (RX interrupt mask)</t>
+  </si>
+  <si>
+    <t>1 = UART fires INTID 33 when a byte arrives in RX FIFO</t>
+  </si>
+  <si>
+    <t>UART_MIS</t>
+  </si>
+  <si>
+    <t>Masked Interrupt Status</t>
+  </si>
+  <si>
+    <t>0x09000040 (QEMU) / 0x40030040 (RPi5)</t>
+  </si>
+  <si>
+    <t>Read in IRQ handler to confirm WHICH UART event caused the interrupt</t>
+  </si>
+  <si>
+    <t>RXMIS</t>
+  </si>
+  <si>
+    <t>1 = RX interrupt is the active source</t>
+  </si>
+  <si>
+    <t>UART_ICR</t>
+  </si>
+  <si>
+    <t>Interrupt Clear Register</t>
+  </si>
+  <si>
+    <t>0x09000044 (QEMU) / 0x40030044 (RPi5)</t>
+  </si>
+  <si>
+    <t>Write 1 to clear a specific pending UART interrupt after handling it</t>
+  </si>
+  <si>
+    <t>RXIC</t>
+  </si>
+  <si>
+    <t>Write (1&lt;&lt;4) to clear RX interrupt; 0x7FF clears all</t>
   </si>
 </sst>
 </file>
@@ -1183,7 +1652,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1211,6 +1680,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1314,7 +1789,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1335,6 +1810,18 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1347,24 +1834,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1374,9 +1843,16 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2626,24 +3102,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="64.2" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>322</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="18" t="s">
         <v>323</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
@@ -3225,127 +3701,127 @@
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="15" t="s">
         <v>324</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="15" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="23" t="s">
         <v>326</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="12" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="23"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="19" t="s">
+      <c r="A19" s="21"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="13" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A20" s="23"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="19" t="s">
+      <c r="A20" s="21"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="13" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="24"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="21" t="s">
+      <c r="A21" s="22"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="14" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="23" t="s">
         <v>331</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="12" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A23" s="23"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="19" t="s">
+      <c r="A23" s="21"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="13" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="24"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="21" t="s">
+      <c r="A24" s="22"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="14" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="23" t="s">
         <v>334</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="12" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A26" s="23"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="19" t="s">
+      <c r="A26" s="21"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="13" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="23"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="19" t="s">
+      <c r="A27" s="21"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="13" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="24"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="21" t="s">
+      <c r="A28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="14" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="12" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A30" s="23"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="19" t="s">
+      <c r="A30" s="21"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="13" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="24"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="21" t="s">
+      <c r="A31" s="22"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="14" t="s">
         <v>343</v>
       </c>
     </row>
@@ -3658,4 +4134,609 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AAF4FB5-1D09-4B64-947B-618607C87C01}">
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="26.88671875" customWidth="1"/>
+    <col min="4" max="4" width="57" customWidth="1"/>
+    <col min="5" max="6" width="21.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>344</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>345</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>346</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>347</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>355</v>
+      </c>
+      <c r="C3" t="s">
+        <v>356</v>
+      </c>
+      <c r="D3" t="s">
+        <v>357</v>
+      </c>
+      <c r="E3" t="s">
+        <v>358</v>
+      </c>
+      <c r="F3" t="s">
+        <v>359</v>
+      </c>
+      <c r="G3" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="26" t="s">
+        <v>361</v>
+      </c>
+      <c r="B4" t="s">
+        <v>362</v>
+      </c>
+      <c r="C4" t="s">
+        <v>363</v>
+      </c>
+      <c r="D4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E4" t="s">
+        <v>365</v>
+      </c>
+      <c r="F4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G4" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="B5" t="s">
+        <v>369</v>
+      </c>
+      <c r="C5" t="s">
+        <v>370</v>
+      </c>
+      <c r="D5" t="s">
+        <v>371</v>
+      </c>
+      <c r="E5" t="s">
+        <v>372</v>
+      </c>
+      <c r="F5" t="s">
+        <v>373</v>
+      </c>
+      <c r="G5" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="B6" t="s">
+        <v>376</v>
+      </c>
+      <c r="C6" t="s">
+        <v>370</v>
+      </c>
+      <c r="D6" t="s">
+        <v>377</v>
+      </c>
+      <c r="E6" t="s">
+        <v>378</v>
+      </c>
+      <c r="F6" t="s">
+        <v>379</v>
+      </c>
+      <c r="G6" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="E7" t="s">
+        <v>381</v>
+      </c>
+      <c r="F7" t="s">
+        <v>366</v>
+      </c>
+      <c r="G7" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="E8" t="s">
+        <v>383</v>
+      </c>
+      <c r="F8" t="s">
+        <v>384</v>
+      </c>
+      <c r="G8" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="26" t="s">
+        <v>386</v>
+      </c>
+      <c r="B9" t="s">
+        <v>387</v>
+      </c>
+      <c r="C9" t="s">
+        <v>388</v>
+      </c>
+      <c r="D9" t="s">
+        <v>389</v>
+      </c>
+      <c r="E9" t="s">
+        <v>390</v>
+      </c>
+      <c r="F9" t="s">
+        <v>373</v>
+      </c>
+      <c r="G9" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="B10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C10" t="s">
+        <v>394</v>
+      </c>
+      <c r="D10" t="s">
+        <v>395</v>
+      </c>
+      <c r="E10" t="s">
+        <v>396</v>
+      </c>
+      <c r="F10" t="s">
+        <v>397</v>
+      </c>
+      <c r="G10" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="26" t="s">
+        <v>399</v>
+      </c>
+      <c r="B11" t="s">
+        <v>400</v>
+      </c>
+      <c r="C11" t="s">
+        <v>401</v>
+      </c>
+      <c r="D11" t="s">
+        <v>402</v>
+      </c>
+      <c r="E11" t="s">
+        <v>403</v>
+      </c>
+      <c r="F11" t="s">
+        <v>404</v>
+      </c>
+      <c r="G11" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="26" t="s">
+        <v>406</v>
+      </c>
+      <c r="B12" t="s">
+        <v>407</v>
+      </c>
+      <c r="C12" t="s">
+        <v>408</v>
+      </c>
+      <c r="D12" t="s">
+        <v>409</v>
+      </c>
+      <c r="E12" t="s">
+        <v>403</v>
+      </c>
+      <c r="F12" t="s">
+        <v>404</v>
+      </c>
+      <c r="G12" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="26" t="s">
+        <v>411</v>
+      </c>
+      <c r="B13" t="s">
+        <v>412</v>
+      </c>
+      <c r="C13" t="s">
+        <v>413</v>
+      </c>
+      <c r="D13" t="s">
+        <v>414</v>
+      </c>
+      <c r="E13" t="s">
+        <v>415</v>
+      </c>
+      <c r="F13" t="s">
+        <v>416</v>
+      </c>
+      <c r="G13" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="26" t="s">
+        <v>418</v>
+      </c>
+      <c r="B14" t="s">
+        <v>419</v>
+      </c>
+      <c r="C14" t="s">
+        <v>420</v>
+      </c>
+      <c r="D14" t="s">
+        <v>421</v>
+      </c>
+      <c r="E14" t="s">
+        <v>415</v>
+      </c>
+      <c r="F14" t="s">
+        <v>422</v>
+      </c>
+      <c r="G14" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="26" t="s">
+        <v>424</v>
+      </c>
+      <c r="B15" t="s">
+        <v>425</v>
+      </c>
+      <c r="C15" t="s">
+        <v>426</v>
+      </c>
+      <c r="D15" t="s">
+        <v>427</v>
+      </c>
+      <c r="E15" t="s">
+        <v>428</v>
+      </c>
+      <c r="F15" t="s">
+        <v>429</v>
+      </c>
+      <c r="G15" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
+        <v>431</v>
+      </c>
+      <c r="B16" t="s">
+        <v>432</v>
+      </c>
+      <c r="C16" t="s">
+        <v>433</v>
+      </c>
+      <c r="D16" t="s">
+        <v>434</v>
+      </c>
+      <c r="E16" t="s">
+        <v>396</v>
+      </c>
+      <c r="F16" t="s">
+        <v>397</v>
+      </c>
+      <c r="G16" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="26" t="s">
+        <v>436</v>
+      </c>
+      <c r="B17" t="s">
+        <v>437</v>
+      </c>
+      <c r="C17" t="s">
+        <v>438</v>
+      </c>
+      <c r="D17" t="s">
+        <v>439</v>
+      </c>
+      <c r="E17" t="s">
+        <v>440</v>
+      </c>
+      <c r="F17" t="s">
+        <v>353</v>
+      </c>
+      <c r="G17" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="26" t="s">
+        <v>442</v>
+      </c>
+      <c r="B18" t="s">
+        <v>443</v>
+      </c>
+      <c r="C18" t="s">
+        <v>444</v>
+      </c>
+      <c r="D18" t="s">
+        <v>445</v>
+      </c>
+      <c r="E18" t="s">
+        <v>446</v>
+      </c>
+      <c r="F18" t="s">
+        <v>447</v>
+      </c>
+      <c r="G18" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="B19" t="s">
+        <v>450</v>
+      </c>
+      <c r="C19" t="s">
+        <v>451</v>
+      </c>
+      <c r="D19" t="s">
+        <v>452</v>
+      </c>
+      <c r="E19" t="s">
+        <v>453</v>
+      </c>
+      <c r="F19" t="s">
+        <v>454</v>
+      </c>
+      <c r="G19" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="E20" t="s">
+        <v>456</v>
+      </c>
+      <c r="F20" t="s">
+        <v>457</v>
+      </c>
+      <c r="G20" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="26" t="s">
+        <v>459</v>
+      </c>
+      <c r="B21" t="s">
+        <v>460</v>
+      </c>
+      <c r="C21" t="s">
+        <v>461</v>
+      </c>
+      <c r="D21" t="s">
+        <v>462</v>
+      </c>
+      <c r="E21" t="s">
+        <v>463</v>
+      </c>
+      <c r="F21" t="s">
+        <v>464</v>
+      </c>
+      <c r="G21" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="26" t="s">
+        <v>466</v>
+      </c>
+      <c r="B22" t="s">
+        <v>467</v>
+      </c>
+      <c r="C22" t="s">
+        <v>468</v>
+      </c>
+      <c r="D22" t="s">
+        <v>469</v>
+      </c>
+      <c r="E22" t="s">
+        <v>470</v>
+      </c>
+      <c r="F22" t="s">
+        <v>353</v>
+      </c>
+      <c r="G22" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="26" t="s">
+        <v>472</v>
+      </c>
+      <c r="B23" t="s">
+        <v>473</v>
+      </c>
+      <c r="C23" t="s">
+        <v>474</v>
+      </c>
+      <c r="D23" t="s">
+        <v>475</v>
+      </c>
+      <c r="E23" t="s">
+        <v>476</v>
+      </c>
+      <c r="F23" t="s">
+        <v>477</v>
+      </c>
+      <c r="G23" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="26" t="s">
+        <v>472</v>
+      </c>
+      <c r="E24" t="s">
+        <v>479</v>
+      </c>
+      <c r="F24" t="s">
+        <v>480</v>
+      </c>
+      <c r="G24" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="26" t="s">
+        <v>482</v>
+      </c>
+      <c r="B25" t="s">
+        <v>483</v>
+      </c>
+      <c r="C25" t="s">
+        <v>484</v>
+      </c>
+      <c r="D25" t="s">
+        <v>485</v>
+      </c>
+      <c r="E25" t="s">
+        <v>486</v>
+      </c>
+      <c r="F25" t="s">
+        <v>477</v>
+      </c>
+      <c r="G25" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="26" t="s">
+        <v>488</v>
+      </c>
+      <c r="B26" t="s">
+        <v>489</v>
+      </c>
+      <c r="C26" t="s">
+        <v>490</v>
+      </c>
+      <c r="D26" t="s">
+        <v>491</v>
+      </c>
+      <c r="E26" t="s">
+        <v>492</v>
+      </c>
+      <c r="F26" t="s">
+        <v>477</v>
+      </c>
+      <c r="G26" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="26" t="s">
+        <v>494</v>
+      </c>
+      <c r="B27" t="s">
+        <v>495</v>
+      </c>
+      <c r="C27" t="s">
+        <v>496</v>
+      </c>
+      <c r="D27" t="s">
+        <v>497</v>
+      </c>
+      <c r="E27" t="s">
+        <v>498</v>
+      </c>
+      <c r="F27" t="s">
+        <v>477</v>
+      </c>
+      <c r="G27" t="s">
+        <v>499</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>